<commit_message>
Added temp and humidity
</commit_message>
<xml_diff>
--- a/SLSS V6/SLSS V6 BoM.xlsx
+++ b/SLSS V6/SLSS V6 BoM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://npluk-my.sharepoint.com/personal/james_edwards_npl_co_uk/Documents/Documents/SLSS/SLSS V6/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Documents\SLSS\SLSS V6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{FBF96A9E-FB1A-4F82-90CC-0F46C2486A3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FBF74107-ED26-4888-B02C-80CAE79B615E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53299886-F7F5-4F11-8640-35745ED59189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{0175BE9B-09DB-4935-9617-04C8C213D07E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{0175BE9B-09DB-4935-9617-04C8C213D07E}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="95">
   <si>
     <t>No</t>
   </si>
@@ -248,15 +248,9 @@
     <t>Wurth Elektronik M3 Standoff, 12 mm Body, 6 mm Stud, Brass</t>
   </si>
   <si>
-    <t xml:space="preserve">SSK-M3-6-A2 </t>
-  </si>
-  <si>
     <t>m3 countersunk</t>
   </si>
   <si>
-    <t>M3 countersunk for battery plate</t>
-  </si>
-  <si>
     <t>3mm ID 5mm OD PVC tubing</t>
   </si>
   <si>
@@ -279,6 +273,54 @@
   </si>
   <si>
     <t>HTBI-M2-BR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SSK-M3-8-A2 </t>
+  </si>
+  <si>
+    <t>M3x8 countersunk</t>
+  </si>
+  <si>
+    <t>Cable gland</t>
+  </si>
+  <si>
+    <t>834-775</t>
+  </si>
+  <si>
+    <t>Rotary encoder</t>
+  </si>
+  <si>
+    <t>?</t>
+  </si>
+  <si>
+    <t>Temp and humidity sensor</t>
+  </si>
+  <si>
+    <t>https://thepihut.com/products/adafruit-sensirion-sht45-precision-temperature-humidity-sensor-stemma-qt-qwiic?_su_rec=gPgvVkC3dW6FfAEJq0881OPq3ij1vB_9ivObglz7OCtLQ4x9CCdThHfIblPWfjWXhaHp-Zus8pchBDixiEBvxtzl42kSFJXCLvApSIxeqGJQjZOxL-qQVXRPFEycGK4nyFUlvQ9d1l4NTvszKXRB66hcvtZM-w7LyzjejeUuSTZvU1BHrcSJX66WPwzqIMBMte3ImXEEsYUXJIT0WVrBMUbtJprp3CR7IZcgfUrcaSDC2_aDX3a5DxLpMvGPp_IZV6Dtk2z_af85Pg&amp;_su_rec_id=6d4cbdf2-c7e9-45e2-b9f7-1df4307d347d-1792449471&amp;variant=54007545102721</t>
+  </si>
+  <si>
+    <t>PI HUT</t>
+  </si>
+  <si>
+    <t>SSCSOR-M2-8-A2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2 Sealing </t>
+  </si>
+  <si>
+    <t>M2 Sealing for SHT45 Temp and humidity sensor</t>
+  </si>
+  <si>
+    <t>SHT45</t>
+  </si>
+  <si>
+    <t>M2 Standoff</t>
+  </si>
+  <si>
+    <t>M2 standoff for SHT45 temp and humidity</t>
+  </si>
+  <si>
+    <t>224-0469</t>
   </si>
 </sst>
 </file>
@@ -693,7 +735,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB3D4A7C-6DC5-428F-8E7D-79698D90EF4B}">
-  <dimension ref="B1:H28"/>
+  <dimension ref="B1:H34"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="16.6328125" customWidth="1"/>
@@ -863,14 +905,14 @@
         <v>36</v>
       </c>
       <c r="D9" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E9">
         <v>1</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H9" t="s">
         <v>32</v>
@@ -1088,16 +1130,16 @@
         <v>18</v>
       </c>
       <c r="C20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D20" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="E20">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="G20" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="H20" t="s">
         <v>50</v>
@@ -1108,13 +1150,13 @@
         <v>19</v>
       </c>
       <c r="C21" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E21">
         <v>1</v>
       </c>
       <c r="G21" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="H21" t="s">
         <v>32</v>
@@ -1125,10 +1167,10 @@
         <v>20</v>
       </c>
       <c r="C22" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G22" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H22" t="s">
         <v>32</v>
@@ -1139,93 +1181,188 @@
         <v>21</v>
       </c>
       <c r="C23" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E23">
         <v>5</v>
       </c>
       <c r="G23" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H23" t="s">
         <v>50</v>
       </c>
     </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B24">
+        <v>22</v>
+      </c>
+      <c r="C24" t="s">
+        <v>81</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="G24" t="s">
+        <v>82</v>
+      </c>
+      <c r="H24" t="s">
+        <v>32</v>
+      </c>
+    </row>
     <row r="25" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B25" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
+      <c r="B25">
+        <v>23</v>
+      </c>
+      <c r="C25" t="s">
+        <v>83</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="G25" t="s">
+        <v>84</v>
+      </c>
+      <c r="H25" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="26" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B26" t="s">
-        <v>0</v>
+      <c r="B26">
+        <v>24</v>
       </c>
       <c r="C26" t="s">
-        <v>1</v>
+        <v>85</v>
       </c>
       <c r="D26" t="s">
+        <v>91</v>
+      </c>
+      <c r="E26">
         <v>2</v>
       </c>
-      <c r="E26" t="s">
-        <v>3</v>
-      </c>
       <c r="F26" t="s">
-        <v>4</v>
-      </c>
-      <c r="G26" t="s">
-        <v>5</v>
+        <v>86</v>
+      </c>
+      <c r="H26" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="27" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B27">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="C27" t="s">
-        <v>8</v>
+        <v>89</v>
       </c>
       <c r="D27" t="s">
-        <v>9</v>
+        <v>90</v>
       </c>
       <c r="E27">
-        <v>1</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>10</v>
+        <v>4</v>
+      </c>
+      <c r="G27" t="s">
+        <v>88</v>
+      </c>
+      <c r="H27" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="28" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B28">
+        <v>26</v>
+      </c>
+      <c r="C28" t="s">
+        <v>92</v>
+      </c>
+      <c r="D28" t="s">
+        <v>93</v>
+      </c>
+      <c r="E28">
+        <v>4</v>
+      </c>
+      <c r="G28" t="s">
+        <v>94</v>
+      </c>
+      <c r="H28" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="31" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B31" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+    </row>
+    <row r="32" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B32" t="s">
+        <v>0</v>
+      </c>
+      <c r="C32" t="s">
+        <v>1</v>
+      </c>
+      <c r="D32" t="s">
         <v>2</v>
       </c>
-      <c r="C28" t="s">
+      <c r="E32" t="s">
+        <v>3</v>
+      </c>
+      <c r="F32" t="s">
+        <v>4</v>
+      </c>
+      <c r="G32" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B33">
+        <v>1</v>
+      </c>
+      <c r="C33" t="s">
+        <v>8</v>
+      </c>
+      <c r="D33" t="s">
+        <v>9</v>
+      </c>
+      <c r="E33">
+        <v>1</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
         <v>12</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D34" t="s">
         <v>13</v>
       </c>
-      <c r="E28">
-        <v>1</v>
-      </c>
-      <c r="F28" s="1" t="s">
+      <c r="E34">
+        <v>1</v>
+      </c>
+      <c r="F34" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G28" s="6">
+      <c r="G34" s="6">
         <v>326</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F27" r:id="rId1" display="https://docs.arduino.cc/resources/pinouts/ABX00028-full-pinout.pdf" xr:uid="{36804345-AEB4-4E7D-9BC7-C81B0111FE34}"/>
-    <hyperlink ref="F28" r:id="rId2" location="technical-details" display="https://www.adafruit.com/product/326 - technical-details" xr:uid="{4DCB4C25-963E-47BD-BBC1-72406EC1CDC3}"/>
+    <hyperlink ref="F33" r:id="rId1" display="https://docs.arduino.cc/resources/pinouts/ABX00028-full-pinout.pdf" xr:uid="{36804345-AEB4-4E7D-9BC7-C81B0111FE34}"/>
+    <hyperlink ref="F34" r:id="rId2" location="technical-details" display="https://www.adafruit.com/product/326 - technical-details" xr:uid="{4DCB4C25-963E-47BD-BBC1-72406EC1CDC3}"/>
     <hyperlink ref="F10" r:id="rId3" display="https://uk.rs-online.com/web/p/battery-holders/1854647" xr:uid="{9521DDEA-38F0-4C9B-93D2-026EF06185F3}"/>
     <hyperlink ref="F13" r:id="rId4" display="https://www.amazon.co.uk/Youmile-Adapter-Interface-Conversion-pinheader/dp/B0C6KB34GZ/ref=sr_1_2_sspa?adgrpid=1175378829251379&amp;dib=eyJ2IjoiMSJ9.4G6Ta0nHdTLEh2FocR_6LAopYVw4r2qMzhRCDT8wuntULpYMdpu6Nx0Be-yz8Bj9e9U26IGfEcWXQyRzuzmArJG2SmYsuic1ec-oTgGdOdXSJYU02rsaO30kc5AMmWBO2ToZD0-HwJQ0kFMAQ_JhSWGUdU_aVZCU3bqjRWrfp9hgZlz6zhLWVtaBsl9FhPPzi88WScDckO5v8_0yqNFwJueiIPTQoT8aGONiikb1_Y4.B15R7p4uyFc5DNnBMFue4rskW8Z0N7_tFr-4B-ExBhk&amp;dib_tag=se&amp;gb=2&amp;hvadid=73461375099874&amp;hvbmt=be&amp;hvdev=c&amp;hvexpln=0&amp;hvlocphy=247141&amp;hvnetw=o&amp;hvocijid=15363587760079059900--&amp;hvqmt=e&amp;hvtargid=kwd-73461312780525%3Aloc-188&amp;hydadcr=13504_1855336&amp;keywords=arduino+micro+sd+card+module&amp;mcid=16b5a40d7175347296a474d6f7b883e3&amp;qid=1786454835&amp;sr=8-2-spons&amp;aref=HuQ1cV2wpw&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9hdGY&amp;psc=1" xr:uid="{89E43225-4AEF-4BE0-8D27-A8DAACFCBDE6}"/>
+    <hyperlink ref="F12" r:id="rId5" xr:uid="{9101D7C0-2B17-464C-B374-CD94E5126C53}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
began design of PCB
</commit_message>
<xml_diff>
--- a/SLSS V6/SLSS V6 BoM.xlsx
+++ b/SLSS V6/SLSS V6 BoM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Documents\SLSS\SLSS V6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1EC9C7B-35EC-4A62-9C5B-38A8B2C89365}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25D163CB-7330-4B31-8D74-8FB67E25B822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{0175BE9B-09DB-4935-9617-04C8C213D07E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="115">
   <si>
     <t>No</t>
   </si>
@@ -363,6 +363,24 @@
   </si>
   <si>
     <t xml:space="preserve">HPN-M2-A2 </t>
+  </si>
+  <si>
+    <t>Pheonix contact 6 way terminal block</t>
+  </si>
+  <si>
+    <t>220-4305</t>
+  </si>
+  <si>
+    <t>Terminal block 6</t>
+  </si>
+  <si>
+    <t>Terminal block 2</t>
+  </si>
+  <si>
+    <t>Pheonix contact 2 way terminal block</t>
+  </si>
+  <si>
+    <t>220-4260</t>
   </si>
 </sst>
 </file>
@@ -777,7 +795,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB3D4A7C-6DC5-428F-8E7D-79698D90EF4B}">
-  <dimension ref="B1:H39"/>
+  <dimension ref="B1:H41"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="16.6328125" customWidth="1"/>
@@ -1485,6 +1503,40 @@
       </c>
       <c r="G39" s="6">
         <v>326</v>
+      </c>
+    </row>
+    <row r="40" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B40">
+        <v>3</v>
+      </c>
+      <c r="C40" t="s">
+        <v>111</v>
+      </c>
+      <c r="D40" t="s">
+        <v>109</v>
+      </c>
+      <c r="E40">
+        <v>3</v>
+      </c>
+      <c r="G40" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="41" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B41">
+        <v>4</v>
+      </c>
+      <c r="C41" t="s">
+        <v>112</v>
+      </c>
+      <c r="D41" t="s">
+        <v>113</v>
+      </c>
+      <c r="E41">
+        <v>1</v>
+      </c>
+      <c r="G41" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>